<commit_message>
refactor: is_prima 뱃지 전면 제거
- Product 모델에서 is_prima 필드 삭제 (migration 0005)
- serializer/view(badges)/admin에서 제거
- 뱃지 관리: is_limited / is_recommended 만 유지
- 백엔드 docs(products/cart) + 설계문서(IA·화면명세서·추적표·정의서 HTML) 반영
- 요구사항정의서.xlsx 원본 3개 셀 수정 후 HTML 재생성

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/KOOM_요구사항정의서.xlsx
+++ b/KOOM_요구사항정의서.xlsx
@@ -914,7 +914,7 @@
       </c>
       <c r="H4" s="12" t="inlineStr">
         <is>
-          <t>필터: 카테고리, mall, is_prima, is_limited, is_recommended
+          <t>필터: 카테고리, mall, is_limited, is_recommended
 정렬: 최신순·가격순·인기순
 표시: 상품명, 썸네일, 원가(KRW), 예상 JPY 환산가, 뱃지, 크롤 상태</t>
         </is>
@@ -1138,7 +1138,7 @@
       </c>
       <c r="D10" s="14" t="inlineStr">
         <is>
-          <t>뱃지 관리 (prima / 한정 / 추천)</t>
+          <t>뱃지 관리 (한정 / 추천)</t>
         </is>
       </c>
       <c r="E10" s="15" t="inlineStr">
@@ -1153,7 +1153,7 @@
       </c>
       <c r="G10" s="12" t="inlineStr">
         <is>
-          <t>상품별로 is_prima, is_limited, is_recommended 뱃지를 Admin에서 ON/OFF한다.</t>
+          <t>상품별로 is_limited, is_recommended 뱃지를 Admin에서 ON/OFF한다.</t>
         </is>
       </c>
       <c r="H10" s="12" t="inlineStr">

</xml_diff>